<commit_message>
falla insercion pag CPT
</commit_message>
<xml_diff>
--- a/excel ejemplo.xlsx
+++ b/excel ejemplo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4eb886068db04012/Escritorio/Programas/programas de redacción de informes/no hechos/redactor informe atencional/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_C31A942ADDCC282F519A59000DB72F886A63FAE1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1639CB42-616A-41E5-A9A7-FC7D570A39AE}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="11_C31A942ADDCC282F519A59000DB72F886A63FAE1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F96AC858-B4FE-4A9E-9AD1-BAF641A0934D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="info" sheetId="1" r:id="rId1"/>
@@ -348,6 +348,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -11930,6 +11934,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E880BCA-9B7B-44CA-B47A-4AE311898D40}">
   <dimension ref="A1:E659"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="11.21875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -11956,10 +11963,10 @@
         <v>1</v>
       </c>
       <c r="C2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1084</v>
       </c>
       <c r="E2" t="s">
         <v>78</v>
@@ -11973,10 +11980,10 @@
         <v>2</v>
       </c>
       <c r="C3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>2069</v>
+        <v>0</v>
       </c>
       <c r="E3" t="s">
         <v>67</v>
@@ -11990,10 +11997,10 @@
         <v>3</v>
       </c>
       <c r="C4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>1820</v>
       </c>
       <c r="E4" t="s">
         <v>67</v>
@@ -12024,10 +12031,10 @@
         <v>5</v>
       </c>
       <c r="C6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>3164</v>
       </c>
       <c r="E6" t="s">
         <v>78</v>
@@ -12041,10 +12048,10 @@
         <v>6</v>
       </c>
       <c r="C7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7">
-        <v>3190</v>
+        <v>0</v>
       </c>
       <c r="E7" t="s">
         <v>78</v>
@@ -12075,10 +12082,10 @@
         <v>8</v>
       </c>
       <c r="C9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9">
-        <v>3768</v>
+        <v>0</v>
       </c>
       <c r="E9" t="s">
         <v>67</v>
@@ -12092,10 +12099,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>6272</v>
       </c>
       <c r="E10" t="s">
         <v>78</v>
@@ -12126,10 +12133,10 @@
         <v>11</v>
       </c>
       <c r="C12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>7076</v>
       </c>
       <c r="E12" t="s">
         <v>78</v>
@@ -12160,10 +12167,10 @@
         <v>13</v>
       </c>
       <c r="C14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>8332</v>
       </c>
       <c r="E14" t="s">
         <v>78</v>
@@ -12197,7 +12204,7 @@
         <v>1</v>
       </c>
       <c r="D16">
-        <v>6285</v>
+        <v>10408</v>
       </c>
       <c r="E16" t="s">
         <v>78</v>
@@ -12262,10 +12269,10 @@
         <v>19</v>
       </c>
       <c r="C20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>13221</v>
       </c>
       <c r="E20" t="s">
         <v>78</v>
@@ -12296,10 +12303,10 @@
         <v>21</v>
       </c>
       <c r="C22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>7583</v>
+        <v>0</v>
       </c>
       <c r="E22" t="s">
         <v>67</v>
@@ -12367,7 +12374,7 @@
         <v>1</v>
       </c>
       <c r="D26">
-        <v>8520</v>
+        <v>18828</v>
       </c>
       <c r="E26" t="s">
         <v>78</v>
@@ -12466,10 +12473,10 @@
         <v>31</v>
       </c>
       <c r="C32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32">
-        <v>9211</v>
+        <v>0</v>
       </c>
       <c r="E32" t="s">
         <v>67</v>
@@ -12551,10 +12558,10 @@
         <v>36</v>
       </c>
       <c r="C37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D37">
-        <v>10493</v>
+        <v>0</v>
       </c>
       <c r="E37" t="s">
         <v>67</v>
@@ -12619,10 +12626,10 @@
         <v>40</v>
       </c>
       <c r="C41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D41">
-        <v>11212</v>
+        <v>0</v>
       </c>
       <c r="E41" t="s">
         <v>78</v>
@@ -12687,10 +12694,10 @@
         <v>44</v>
       </c>
       <c r="C45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D45">
-        <v>13100</v>
+        <v>0</v>
       </c>
       <c r="E45" t="s">
         <v>67</v>
@@ -12721,10 +12728,10 @@
         <v>46</v>
       </c>
       <c r="C47" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D47">
-        <v>14559</v>
+        <v>0</v>
       </c>
       <c r="E47" t="s">
         <v>78</v>
@@ -12772,10 +12779,10 @@
         <v>2</v>
       </c>
       <c r="C50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D50">
-        <v>0</v>
+        <v>3383</v>
       </c>
       <c r="E50" t="s">
         <v>78</v>
@@ -12823,10 +12830,10 @@
         <v>5</v>
       </c>
       <c r="C53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D53">
-        <v>0</v>
+        <v>5267</v>
       </c>
       <c r="E53" t="s">
         <v>78</v>
@@ -12874,10 +12881,10 @@
         <v>8</v>
       </c>
       <c r="C56" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D56">
-        <v>0</v>
+        <v>7331</v>
       </c>
       <c r="E56" t="s">
         <v>78</v>
@@ -12959,10 +12966,10 @@
         <v>13</v>
       </c>
       <c r="C61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D61">
-        <v>0</v>
+        <v>10875</v>
       </c>
       <c r="E61" t="s">
         <v>78</v>
@@ -12976,10 +12983,10 @@
         <v>14</v>
       </c>
       <c r="C62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D62">
-        <v>0</v>
+        <v>13019</v>
       </c>
       <c r="E62" t="s">
         <v>78</v>
@@ -13027,10 +13034,10 @@
         <v>17</v>
       </c>
       <c r="C65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D65">
-        <v>0</v>
+        <v>14303</v>
       </c>
       <c r="E65" t="s">
         <v>67</v>
@@ -13061,10 +13068,10 @@
         <v>19</v>
       </c>
       <c r="C67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D67">
-        <v>0</v>
+        <v>15823</v>
       </c>
       <c r="E67" t="s">
         <v>78</v>
@@ -13095,10 +13102,10 @@
         <v>21</v>
       </c>
       <c r="C69" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D69">
-        <v>0</v>
+        <v>18067</v>
       </c>
       <c r="E69" t="s">
         <v>78</v>
@@ -13129,10 +13136,10 @@
         <v>23</v>
       </c>
       <c r="C71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D71">
-        <v>0</v>
+        <v>19459</v>
       </c>
       <c r="E71" t="s">
         <v>78</v>
@@ -13605,10 +13612,10 @@
         <v>4</v>
       </c>
       <c r="C99" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D99">
-        <v>0</v>
+        <v>3158</v>
       </c>
       <c r="E99" t="s">
         <v>78</v>
@@ -13656,10 +13663,10 @@
         <v>7</v>
       </c>
       <c r="C102" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D102">
-        <v>0</v>
+        <v>4342</v>
       </c>
       <c r="E102" t="s">
         <v>78</v>
@@ -13690,10 +13697,10 @@
         <v>9</v>
       </c>
       <c r="C104" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D104">
-        <v>0</v>
+        <v>5598</v>
       </c>
       <c r="E104" t="s">
         <v>78</v>
@@ -13758,10 +13765,10 @@
         <v>13</v>
       </c>
       <c r="C108" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D108">
-        <v>0</v>
+        <v>7186</v>
       </c>
       <c r="E108" t="s">
         <v>78</v>
@@ -13809,10 +13816,10 @@
         <v>16</v>
       </c>
       <c r="C111" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D111">
-        <v>0</v>
+        <v>8674</v>
       </c>
       <c r="E111" t="s">
         <v>78</v>
@@ -13843,10 +13850,10 @@
         <v>18</v>
       </c>
       <c r="C113" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D113">
-        <v>0</v>
+        <v>9734</v>
       </c>
       <c r="E113" t="s">
         <v>78</v>
@@ -13894,10 +13901,10 @@
         <v>21</v>
       </c>
       <c r="C116" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D116">
-        <v>0</v>
+        <v>11782</v>
       </c>
       <c r="E116" t="s">
         <v>78</v>
@@ -13928,10 +13935,10 @@
         <v>23</v>
       </c>
       <c r="C118" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D118">
-        <v>0</v>
+        <v>12682</v>
       </c>
       <c r="E118" t="s">
         <v>78</v>
@@ -14013,10 +14020,10 @@
         <v>28</v>
       </c>
       <c r="C123" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D123">
-        <v>0</v>
+        <v>16142</v>
       </c>
       <c r="E123" t="s">
         <v>78</v>
@@ -14359,7 +14366,7 @@
         <v>0</v>
       </c>
       <c r="E143" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.3">
@@ -14421,13 +14428,13 @@
         <v>5</v>
       </c>
       <c r="C147" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D147">
-        <v>0</v>
+        <v>4055</v>
       </c>
       <c r="E147" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.3">
@@ -14444,7 +14451,7 @@
         <v>0</v>
       </c>
       <c r="E148" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.3">
@@ -14489,13 +14496,13 @@
         <v>9</v>
       </c>
       <c r="C151" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D151">
-        <v>0</v>
+        <v>5335</v>
       </c>
       <c r="E151" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.3">
@@ -14523,13 +14530,13 @@
         <v>11</v>
       </c>
       <c r="C153" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D153">
-        <v>0</v>
+        <v>6200</v>
       </c>
       <c r="E153" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.3">
@@ -14546,7 +14553,7 @@
         <v>0</v>
       </c>
       <c r="E154" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.3">
@@ -14557,13 +14564,13 @@
         <v>13</v>
       </c>
       <c r="C155" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D155">
-        <v>0</v>
+        <v>6955</v>
       </c>
       <c r="E155" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.3">
@@ -14591,13 +14598,13 @@
         <v>15</v>
       </c>
       <c r="C157" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D157">
-        <v>0</v>
+        <v>8139</v>
       </c>
       <c r="E157" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.3">
@@ -14665,7 +14672,7 @@
         <v>0</v>
       </c>
       <c r="E161" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.3">
@@ -14750,7 +14757,7 @@
         <v>0</v>
       </c>
       <c r="E166" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.3">
@@ -14767,7 +14774,7 @@
         <v>0</v>
       </c>
       <c r="E167" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.3">
@@ -14801,7 +14808,7 @@
         <v>0</v>
       </c>
       <c r="E169" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.3">
@@ -14829,13 +14836,13 @@
         <v>29</v>
       </c>
       <c r="C171" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D171">
-        <v>0</v>
+        <v>15227</v>
       </c>
       <c r="E171" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.3">
@@ -14903,7 +14910,7 @@
         <v>0</v>
       </c>
       <c r="E175" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.3">
@@ -14914,13 +14921,13 @@
         <v>34</v>
       </c>
       <c r="C176" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D176">
-        <v>0</v>
+        <v>17518</v>
       </c>
       <c r="E176" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.3">
@@ -14965,13 +14972,13 @@
         <v>37</v>
       </c>
       <c r="C179" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D179">
-        <v>0</v>
+        <v>18495</v>
       </c>
       <c r="E179" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.3">
@@ -14988,7 +14995,7 @@
         <v>0</v>
       </c>
       <c r="E180" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.3">
@@ -15022,7 +15029,7 @@
         <v>0</v>
       </c>
       <c r="E182" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.3">
@@ -15073,7 +15080,7 @@
         <v>0</v>
       </c>
       <c r="E185" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.3">
@@ -15107,7 +15114,7 @@
         <v>0</v>
       </c>
       <c r="E187" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.3">
@@ -15124,7 +15131,7 @@
         <v>0</v>
       </c>
       <c r="E188" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.3">
@@ -15169,10 +15176,10 @@
         <v>2</v>
       </c>
       <c r="C191" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D191">
-        <v>0</v>
+        <v>4516</v>
       </c>
       <c r="E191" t="s">
         <v>78</v>
@@ -15243,7 +15250,7 @@
         <v>0</v>
       </c>
       <c r="E195" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.3">
@@ -15271,13 +15278,13 @@
         <v>8</v>
       </c>
       <c r="C197" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D197">
-        <v>0</v>
+        <v>7272</v>
       </c>
       <c r="E197" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.3">
@@ -15294,7 +15301,7 @@
         <v>0</v>
       </c>
       <c r="E198" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.3">
@@ -15328,7 +15335,7 @@
         <v>0</v>
       </c>
       <c r="E200" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.3">
@@ -15345,7 +15352,7 @@
         <v>0</v>
       </c>
       <c r="E201" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.3">
@@ -15379,7 +15386,7 @@
         <v>0</v>
       </c>
       <c r="E203" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.3">
@@ -15396,7 +15403,7 @@
         <v>0</v>
       </c>
       <c r="E204" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.3">
@@ -15413,7 +15420,7 @@
         <v>0</v>
       </c>
       <c r="E205" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.3">
@@ -15458,10 +15465,10 @@
         <v>19</v>
       </c>
       <c r="C208" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D208">
-        <v>0</v>
+        <v>12432</v>
       </c>
       <c r="E208" t="s">
         <v>78</v>
@@ -15498,7 +15505,7 @@
         <v>0</v>
       </c>
       <c r="E210" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.3">
@@ -15532,7 +15539,7 @@
         <v>0</v>
       </c>
       <c r="E212" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.3">
@@ -15543,10 +15550,10 @@
         <v>24</v>
       </c>
       <c r="C213" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D213">
-        <v>0</v>
+        <v>14340</v>
       </c>
       <c r="E213" t="s">
         <v>78</v>
@@ -15566,7 +15573,7 @@
         <v>0</v>
       </c>
       <c r="E214" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.3">
@@ -15600,7 +15607,7 @@
         <v>0</v>
       </c>
       <c r="E216" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.3">
@@ -15651,7 +15658,7 @@
         <v>0</v>
       </c>
       <c r="E219" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="220" spans="1:5" x14ac:dyDescent="0.3">
@@ -15719,7 +15726,7 @@
         <v>0</v>
       </c>
       <c r="E223" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.3">
@@ -15736,7 +15743,7 @@
         <v>0</v>
       </c>
       <c r="E224" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.3">
@@ -15787,7 +15794,7 @@
         <v>0</v>
       </c>
       <c r="E227" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="228" spans="1:5" x14ac:dyDescent="0.3">
@@ -15804,7 +15811,7 @@
         <v>0</v>
       </c>
       <c r="E228" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="229" spans="1:5" x14ac:dyDescent="0.3">
@@ -15815,10 +15822,10 @@
         <v>40</v>
       </c>
       <c r="C229" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D229">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="E229" t="s">
         <v>78</v>
@@ -15838,7 +15845,7 @@
         <v>0</v>
       </c>
       <c r="E230" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="231" spans="1:5" x14ac:dyDescent="0.3">
@@ -15855,7 +15862,7 @@
         <v>0</v>
       </c>
       <c r="E231" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="232" spans="1:5" x14ac:dyDescent="0.3">
@@ -15872,7 +15879,7 @@
         <v>0</v>
       </c>
       <c r="E232" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="233" spans="1:5" x14ac:dyDescent="0.3">
@@ -15889,7 +15896,7 @@
         <v>0</v>
       </c>
       <c r="E233" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="234" spans="1:5" x14ac:dyDescent="0.3">
@@ -15906,7 +15913,7 @@
         <v>0</v>
       </c>
       <c r="E234" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.3">
@@ -15940,7 +15947,7 @@
         <v>0</v>
       </c>
       <c r="E236" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="237" spans="1:5" x14ac:dyDescent="0.3">
@@ -15985,10 +15992,10 @@
         <v>3</v>
       </c>
       <c r="C239" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D239">
-        <v>0</v>
+        <v>3829</v>
       </c>
       <c r="E239" t="s">
         <v>78</v>
@@ -16002,10 +16009,10 @@
         <v>4</v>
       </c>
       <c r="C240" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D240">
-        <v>0</v>
+        <v>5348</v>
       </c>
       <c r="E240" t="s">
         <v>78</v>
@@ -16053,10 +16060,10 @@
         <v>7</v>
       </c>
       <c r="C243" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D243">
-        <v>0</v>
+        <v>6488</v>
       </c>
       <c r="E243" t="s">
         <v>78</v>
@@ -16087,10 +16094,10 @@
         <v>9</v>
       </c>
       <c r="C245" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D245">
-        <v>0</v>
+        <v>8440</v>
       </c>
       <c r="E245" t="s">
         <v>78</v>
@@ -16155,10 +16162,10 @@
         <v>13</v>
       </c>
       <c r="C249" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D249">
-        <v>0</v>
+        <v>10028</v>
       </c>
       <c r="E249" t="s">
         <v>78</v>
@@ -16206,10 +16213,10 @@
         <v>16</v>
       </c>
       <c r="C252" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D252">
-        <v>0</v>
+        <v>11388</v>
       </c>
       <c r="E252" t="s">
         <v>78</v>
@@ -16240,10 +16247,10 @@
         <v>18</v>
       </c>
       <c r="C254" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D254">
-        <v>0</v>
+        <v>12352</v>
       </c>
       <c r="E254" t="s">
         <v>78</v>
@@ -16291,10 +16298,10 @@
         <v>21</v>
       </c>
       <c r="C257" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D257">
-        <v>0</v>
+        <v>14192</v>
       </c>
       <c r="E257" t="s">
         <v>78</v>
@@ -16325,10 +16332,10 @@
         <v>23</v>
       </c>
       <c r="C259" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D259">
-        <v>0</v>
+        <v>15748</v>
       </c>
       <c r="E259" t="s">
         <v>78</v>
@@ -16376,10 +16383,10 @@
         <v>26</v>
       </c>
       <c r="C262" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D262">
-        <v>0</v>
+        <v>18228</v>
       </c>
       <c r="E262" t="s">
         <v>78</v>
@@ -16410,10 +16417,10 @@
         <v>28</v>
       </c>
       <c r="C264" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D264">
-        <v>0</v>
+        <v>19600</v>
       </c>
       <c r="E264" t="s">
         <v>78</v>
@@ -16750,10 +16757,10 @@
         <v>1</v>
       </c>
       <c r="C284" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D284">
-        <v>0</v>
+        <v>1777</v>
       </c>
       <c r="E284" t="s">
         <v>78</v>
@@ -16818,10 +16825,10 @@
         <v>5</v>
       </c>
       <c r="C288" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D288">
-        <v>0</v>
+        <v>4397</v>
       </c>
       <c r="E288" t="s">
         <v>78</v>
@@ -16886,10 +16893,10 @@
         <v>9</v>
       </c>
       <c r="C292" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D292">
-        <v>0</v>
+        <v>6045</v>
       </c>
       <c r="E292" t="s">
         <v>78</v>
@@ -16920,10 +16927,10 @@
         <v>11</v>
       </c>
       <c r="C294" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D294">
-        <v>0</v>
+        <v>7409</v>
       </c>
       <c r="E294" t="s">
         <v>78</v>
@@ -16954,10 +16961,10 @@
         <v>13</v>
       </c>
       <c r="C296" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D296">
-        <v>0</v>
+        <v>8433</v>
       </c>
       <c r="E296" t="s">
         <v>78</v>
@@ -16988,10 +16995,10 @@
         <v>15</v>
       </c>
       <c r="C298" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D298">
-        <v>0</v>
+        <v>9953</v>
       </c>
       <c r="E298" t="s">
         <v>78</v>
@@ -17073,10 +17080,10 @@
         <v>20</v>
       </c>
       <c r="C303" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D303">
-        <v>0</v>
+        <v>12349</v>
       </c>
       <c r="E303" t="s">
         <v>67</v>
@@ -17141,10 +17148,10 @@
         <v>24</v>
       </c>
       <c r="C307" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D307">
-        <v>0</v>
+        <v>14977</v>
       </c>
       <c r="E307" t="s">
         <v>78</v>
@@ -17158,10 +17165,10 @@
         <v>25</v>
       </c>
       <c r="C308" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D308">
-        <v>0</v>
+        <v>16265</v>
       </c>
       <c r="E308" t="s">
         <v>78</v>
@@ -17192,10 +17199,10 @@
         <v>27</v>
       </c>
       <c r="C310" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D310">
-        <v>0</v>
+        <v>17277</v>
       </c>
       <c r="E310" t="s">
         <v>78</v>
@@ -17226,10 +17233,10 @@
         <v>29</v>
       </c>
       <c r="C312" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D312">
-        <v>0</v>
+        <v>19409</v>
       </c>
       <c r="E312" t="s">
         <v>78</v>
@@ -17566,10 +17573,10 @@
         <v>2</v>
       </c>
       <c r="C332" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D332">
-        <v>0</v>
+        <v>1835</v>
       </c>
       <c r="E332" t="s">
         <v>78</v>
@@ -17668,10 +17675,10 @@
         <v>8</v>
       </c>
       <c r="C338" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D338">
-        <v>0</v>
+        <v>5586</v>
       </c>
       <c r="E338" t="s">
         <v>78</v>
@@ -17753,10 +17760,10 @@
         <v>13</v>
       </c>
       <c r="C343" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D343">
-        <v>0</v>
+        <v>8273</v>
       </c>
       <c r="E343" t="s">
         <v>78</v>
@@ -17804,10 +17811,10 @@
         <v>16</v>
       </c>
       <c r="C346" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D346">
-        <v>0</v>
+        <v>9670</v>
       </c>
       <c r="E346" t="s">
         <v>78</v>
@@ -17855,10 +17862,10 @@
         <v>19</v>
       </c>
       <c r="C349" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D349">
-        <v>0</v>
+        <v>11166</v>
       </c>
       <c r="E349" t="s">
         <v>78</v>
@@ -17889,10 +17896,10 @@
         <v>21</v>
       </c>
       <c r="C351" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D351">
-        <v>0</v>
+        <v>12417</v>
       </c>
       <c r="E351" t="s">
         <v>78</v>
@@ -17923,10 +17930,10 @@
         <v>23</v>
       </c>
       <c r="C353" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D353">
-        <v>0</v>
+        <v>13970</v>
       </c>
       <c r="E353" t="s">
         <v>78</v>
@@ -17940,10 +17947,10 @@
         <v>24</v>
       </c>
       <c r="C354" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D354">
-        <v>0</v>
+        <v>14812</v>
       </c>
       <c r="E354" t="s">
         <v>78</v>
@@ -18025,10 +18032,10 @@
         <v>29</v>
       </c>
       <c r="C359" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D359">
-        <v>0</v>
+        <v>17514</v>
       </c>
       <c r="E359" t="s">
         <v>78</v>
@@ -18042,10 +18049,10 @@
         <v>30</v>
       </c>
       <c r="C360" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D360">
-        <v>0</v>
+        <v>19594</v>
       </c>
       <c r="E360" t="s">
         <v>78</v>
@@ -18382,10 +18389,10 @@
         <v>3</v>
       </c>
       <c r="C380" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D380">
-        <v>0</v>
+        <v>3636</v>
       </c>
       <c r="E380" t="s">
         <v>78</v>
@@ -18399,10 +18406,10 @@
         <v>4</v>
       </c>
       <c r="C381" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D381">
-        <v>0</v>
+        <v>4195</v>
       </c>
       <c r="E381" t="s">
         <v>78</v>
@@ -18450,10 +18457,10 @@
         <v>7</v>
       </c>
       <c r="C384" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D384">
-        <v>0</v>
+        <v>5779</v>
       </c>
       <c r="E384" t="s">
         <v>78</v>
@@ -18484,10 +18491,10 @@
         <v>9</v>
       </c>
       <c r="C386" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D386">
-        <v>0</v>
+        <v>6839</v>
       </c>
       <c r="E386" t="s">
         <v>78</v>
@@ -18552,10 +18559,10 @@
         <v>13</v>
       </c>
       <c r="C390" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D390">
-        <v>0</v>
+        <v>8711</v>
       </c>
       <c r="E390" t="s">
         <v>78</v>
@@ -18603,10 +18610,10 @@
         <v>16</v>
       </c>
       <c r="C393" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D393">
-        <v>0</v>
+        <v>10555</v>
       </c>
       <c r="E393" t="s">
         <v>78</v>
@@ -18637,10 +18644,10 @@
         <v>18</v>
       </c>
       <c r="C395" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D395">
-        <v>0</v>
+        <v>12483</v>
       </c>
       <c r="E395" t="s">
         <v>78</v>
@@ -18671,10 +18678,10 @@
         <v>20</v>
       </c>
       <c r="C397" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D397">
-        <v>0</v>
+        <v>14687</v>
       </c>
       <c r="E397" t="s">
         <v>67</v>
@@ -18722,10 +18729,10 @@
         <v>23</v>
       </c>
       <c r="C400" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D400">
-        <v>0</v>
+        <v>16979</v>
       </c>
       <c r="E400" t="s">
         <v>78</v>
@@ -18773,10 +18780,10 @@
         <v>26</v>
       </c>
       <c r="C403" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D403">
-        <v>0</v>
+        <v>18943</v>
       </c>
       <c r="E403" t="s">
         <v>78</v>
@@ -19147,10 +19154,10 @@
         <v>1</v>
       </c>
       <c r="C425" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D425">
-        <v>0</v>
+        <v>3159</v>
       </c>
       <c r="E425" t="s">
         <v>78</v>
@@ -19215,10 +19222,10 @@
         <v>5</v>
       </c>
       <c r="C429" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D429">
-        <v>0</v>
+        <v>6507</v>
       </c>
       <c r="E429" t="s">
         <v>78</v>
@@ -19317,10 +19324,10 @@
         <v>11</v>
       </c>
       <c r="C435" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D435">
-        <v>0</v>
+        <v>8504</v>
       </c>
       <c r="E435" t="s">
         <v>78</v>
@@ -19351,10 +19358,10 @@
         <v>13</v>
       </c>
       <c r="C437" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D437">
-        <v>0</v>
+        <v>10311</v>
       </c>
       <c r="E437" t="s">
         <v>78</v>
@@ -19385,10 +19392,10 @@
         <v>15</v>
       </c>
       <c r="C439" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D439">
-        <v>0</v>
+        <v>11868</v>
       </c>
       <c r="E439" t="s">
         <v>78</v>
@@ -19453,10 +19460,10 @@
         <v>19</v>
       </c>
       <c r="C443" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D443">
-        <v>0</v>
+        <v>13807</v>
       </c>
       <c r="E443" t="s">
         <v>78</v>
@@ -19612,7 +19619,7 @@
         <v>0</v>
       </c>
       <c r="E452" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="453" spans="1:5" x14ac:dyDescent="0.3">
@@ -19623,13 +19630,13 @@
         <v>29</v>
       </c>
       <c r="C453" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D453">
-        <v>0</v>
+        <v>18091</v>
       </c>
       <c r="E453" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="454" spans="1:5" x14ac:dyDescent="0.3">
@@ -19963,10 +19970,10 @@
         <v>2</v>
       </c>
       <c r="C473" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D473">
-        <v>0</v>
+        <v>2425</v>
       </c>
       <c r="E473" t="s">
         <v>78</v>
@@ -20065,10 +20072,10 @@
         <v>8</v>
       </c>
       <c r="C479" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D479">
-        <v>0</v>
+        <v>6504</v>
       </c>
       <c r="E479" t="s">
         <v>78</v>
@@ -20150,10 +20157,10 @@
         <v>13</v>
       </c>
       <c r="C484" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D484">
-        <v>0</v>
+        <v>12042</v>
       </c>
       <c r="E484" t="s">
         <v>78</v>
@@ -20167,10 +20174,10 @@
         <v>14</v>
       </c>
       <c r="C485" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D485">
-        <v>0</v>
+        <v>11301</v>
       </c>
       <c r="E485" t="s">
         <v>78</v>
@@ -20201,10 +20208,10 @@
         <v>16</v>
       </c>
       <c r="C487" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D487">
-        <v>0</v>
+        <v>13642</v>
       </c>
       <c r="E487" t="s">
         <v>78</v>
@@ -20320,10 +20327,10 @@
         <v>23</v>
       </c>
       <c r="C494" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D494">
-        <v>0</v>
+        <v>16509</v>
       </c>
       <c r="E494" t="s">
         <v>78</v>
@@ -20337,10 +20344,10 @@
         <v>24</v>
       </c>
       <c r="C495" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D495">
-        <v>0</v>
+        <v>18561</v>
       </c>
       <c r="E495" t="s">
         <v>78</v>
@@ -20779,10 +20786,10 @@
         <v>3</v>
       </c>
       <c r="C521" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D521">
-        <v>0</v>
+        <v>2609</v>
       </c>
       <c r="E521" t="s">
         <v>78</v>
@@ -20796,10 +20803,10 @@
         <v>4</v>
       </c>
       <c r="C522" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D522">
-        <v>0</v>
+        <v>3649</v>
       </c>
       <c r="E522" t="s">
         <v>78</v>
@@ -20847,10 +20854,10 @@
         <v>7</v>
       </c>
       <c r="C525" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D525">
-        <v>0</v>
+        <v>5909</v>
       </c>
       <c r="E525" t="s">
         <v>78</v>
@@ -20881,10 +20888,10 @@
         <v>9</v>
       </c>
       <c r="C527" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D527">
-        <v>0</v>
+        <v>7625</v>
       </c>
       <c r="E527" t="s">
         <v>78</v>
@@ -20949,10 +20956,10 @@
         <v>13</v>
       </c>
       <c r="C531" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D531">
-        <v>0</v>
+        <v>8985</v>
       </c>
       <c r="E531" t="s">
         <v>78</v>
@@ -20966,10 +20973,10 @@
         <v>14</v>
       </c>
       <c r="C532" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D532">
-        <v>0</v>
+        <v>10637</v>
       </c>
       <c r="E532" t="s">
         <v>78</v>
@@ -21000,10 +21007,10 @@
         <v>16</v>
       </c>
       <c r="C534" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D534">
-        <v>0</v>
+        <v>14066</v>
       </c>
       <c r="E534" t="s">
         <v>78</v>
@@ -21034,10 +21041,10 @@
         <v>18</v>
       </c>
       <c r="C536" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D536">
-        <v>0</v>
+        <v>12994</v>
       </c>
       <c r="E536" t="s">
         <v>78</v>
@@ -21085,10 +21092,10 @@
         <v>21</v>
       </c>
       <c r="C539" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D539">
-        <v>0</v>
+        <v>17238</v>
       </c>
       <c r="E539" t="s">
         <v>78</v>
@@ -21119,10 +21126,10 @@
         <v>23</v>
       </c>
       <c r="C541" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D541">
-        <v>0</v>
+        <v>18549</v>
       </c>
       <c r="E541" t="s">
         <v>78</v>
@@ -21544,10 +21551,10 @@
         <v>1</v>
       </c>
       <c r="C566" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D566">
-        <v>0</v>
+        <v>3447</v>
       </c>
       <c r="E566" t="s">
         <v>78</v>
@@ -21612,10 +21619,10 @@
         <v>5</v>
       </c>
       <c r="C570" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D570">
-        <v>0</v>
+        <v>5035</v>
       </c>
       <c r="E570" t="s">
         <v>78</v>
@@ -21629,10 +21636,10 @@
         <v>6</v>
       </c>
       <c r="C571" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D571">
-        <v>0</v>
+        <v>7563</v>
       </c>
       <c r="E571" t="s">
         <v>78</v>
@@ -21680,10 +21687,10 @@
         <v>9</v>
       </c>
       <c r="C574" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D574">
-        <v>0</v>
+        <v>9352</v>
       </c>
       <c r="E574" t="s">
         <v>78</v>
@@ -21714,10 +21721,10 @@
         <v>11</v>
       </c>
       <c r="C576" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D576">
-        <v>0</v>
+        <v>10935</v>
       </c>
       <c r="E576" t="s">
         <v>78</v>
@@ -21731,10 +21738,10 @@
         <v>12</v>
       </c>
       <c r="C577" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D577">
-        <v>0</v>
+        <v>11867</v>
       </c>
       <c r="E577" t="s">
         <v>78</v>
@@ -21748,10 +21755,10 @@
         <v>13</v>
       </c>
       <c r="C578" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D578">
-        <v>0</v>
+        <v>13707</v>
       </c>
       <c r="E578" t="s">
         <v>78</v>
@@ -21782,10 +21789,10 @@
         <v>15</v>
       </c>
       <c r="C580" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D580">
-        <v>0</v>
+        <v>15328</v>
       </c>
       <c r="E580" t="s">
         <v>78</v>
@@ -21850,10 +21857,10 @@
         <v>19</v>
       </c>
       <c r="C584" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D584">
-        <v>0</v>
+        <v>17731</v>
       </c>
       <c r="E584" t="s">
         <v>78</v>
@@ -22360,10 +22367,10 @@
         <v>2</v>
       </c>
       <c r="C614" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D614">
-        <v>0</v>
+        <v>2273</v>
       </c>
       <c r="E614" t="s">
         <v>78</v>
@@ -22411,10 +22418,10 @@
         <v>5</v>
       </c>
       <c r="C617" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D617">
-        <v>0</v>
+        <v>4429</v>
       </c>
       <c r="E617" t="s">
         <v>78</v>
@@ -22462,10 +22469,10 @@
         <v>8</v>
       </c>
       <c r="C620" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D620">
-        <v>0</v>
+        <v>7337</v>
       </c>
       <c r="E620" t="s">
         <v>78</v>
@@ -22547,10 +22554,10 @@
         <v>13</v>
       </c>
       <c r="C625" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D625">
-        <v>0</v>
+        <v>11574</v>
       </c>
       <c r="E625" t="s">
         <v>78</v>
@@ -22564,10 +22571,10 @@
         <v>14</v>
       </c>
       <c r="C626" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D626">
-        <v>0</v>
+        <v>10998</v>
       </c>
       <c r="E626" t="s">
         <v>78</v>
@@ -22598,10 +22605,10 @@
         <v>16</v>
       </c>
       <c r="C628" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D628">
-        <v>0</v>
+        <v>12753</v>
       </c>
       <c r="E628" t="s">
         <v>78</v>
@@ -22649,10 +22656,10 @@
         <v>19</v>
       </c>
       <c r="C631" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D631">
-        <v>0</v>
+        <v>15710</v>
       </c>
       <c r="E631" t="s">
         <v>78</v>
@@ -22683,10 +22690,10 @@
         <v>21</v>
       </c>
       <c r="C633" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D633">
-        <v>0</v>
+        <v>17309</v>
       </c>
       <c r="E633" t="s">
         <v>78</v>
@@ -22717,10 +22724,10 @@
         <v>23</v>
       </c>
       <c r="C635" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D635">
-        <v>0</v>
+        <v>18753</v>
       </c>
       <c r="E635" t="s">
         <v>78</v>
@@ -22734,10 +22741,10 @@
         <v>24</v>
       </c>
       <c r="C636" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D636">
-        <v>0</v>
+        <v>19250</v>
       </c>
       <c r="E636" t="s">
         <v>78</v>

</xml_diff>